<commit_message>
updated to use target instead of normname
</commit_message>
<xml_diff>
--- a/stimuli/660CorpusMasterSheet.xlsx
+++ b/stimuli/660CorpusMasterSheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bowdoin-my.sharepoint.com/personal/c_hambric_bowdoin_edu/Documents/Documents/Blocked_Practice/stimuli/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f8df46a41a7bbc33/Research/Blocked_Practice/stimuli/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="12" documentId="8_{9A1B9D56-DE9B-714E-A0ED-61EE4E9F4BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CAB7461-9D05-4EC8-BF56-59073057CCEA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F272CC09-A90E-7241-817B-293133178CF1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{F272CC09-A90E-7241-817B-293133178CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13267,7 +13267,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13278,7 +13278,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13288,7 +13288,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13351,7 +13351,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13362,7 +13362,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13372,7 +13372,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13435,7 +13435,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13446,7 +13446,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13456,7 +13456,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13519,7 +13519,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13530,7 +13530,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13540,7 +13540,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13603,7 +13603,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13614,7 +13614,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13624,7 +13624,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13687,7 +13687,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13698,7 +13698,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13708,7 +13708,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13771,7 +13771,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13782,7 +13782,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13792,7 +13792,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13855,7 +13855,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13866,7 +13866,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13876,7 +13876,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -13939,7 +13939,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -13950,7 +13950,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -13960,7 +13960,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14023,7 +14023,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14034,7 +14034,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14044,7 +14044,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14107,7 +14107,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14118,7 +14118,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14128,7 +14128,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14191,7 +14191,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14202,7 +14202,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14212,7 +14212,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14275,7 +14275,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14286,7 +14286,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14296,7 +14296,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14359,7 +14359,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14370,7 +14370,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14380,7 +14380,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14443,7 +14443,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14454,7 +14454,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14464,7 +14464,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14527,7 +14527,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14538,7 +14538,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14548,7 +14548,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14611,7 +14611,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14622,7 +14622,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14632,7 +14632,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14695,7 +14695,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14706,7 +14706,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14716,7 +14716,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14779,7 +14779,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14790,7 +14790,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14800,7 +14800,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14863,7 +14863,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14874,7 +14874,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14884,7 +14884,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -14947,7 +14947,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -14958,7 +14958,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -14968,7 +14968,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15031,7 +15031,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -15042,7 +15042,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -15052,7 +15052,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15115,7 +15115,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -15126,7 +15126,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -15136,7 +15136,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15199,7 +15199,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -15210,7 +15210,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -15220,7 +15220,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15283,7 +15283,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -15294,7 +15294,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -15304,7 +15304,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15367,7 +15367,7 @@
         <a:effectLst/>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:blipFill dpi="0" rotWithShape="0">
                 <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
                 <a:srcRect/>
@@ -15378,7 +15378,7 @@
             </a14:hiddenFill>
           </a:ext>
           <a:ext uri="{91240B29-F687-4f45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525" cap="flat">
+            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="" w="9525" cap="flat">
               <a:solidFill>
                 <a:srgbClr val="808080"/>
               </a:solidFill>
@@ -15388,7 +15388,7 @@
             </a14:hiddenLine>
           </a:ext>
           <a:ext uri="{AF507438-7753-43e0-B8FC-AC1667EBCBE1}">
-            <a14:hiddenEffects xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+            <a14:hiddenEffects xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
               <a:effectLst>
                 <a:outerShdw blurRad="63500" dist="38099" dir="2700000" algn="ctr" rotWithShape="0">
                   <a:srgbClr val="000000">
@@ -15404,10 +15404,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -15728,11 +15724,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21C205F-EF89-204A-A1A4-B93CBBED4F55}">
   <dimension ref="A1:AB661"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="11.125" customWidth="1"/>
-    <col min="2" max="2" width="22.375" customWidth="1"/>
-    <col min="3" max="25" width="11.125" customWidth="1"/>
+    <col min="1" max="1" width="11.08203125" customWidth="1"/>
+    <col min="2" max="2" width="22.33203125" customWidth="1"/>
+    <col min="3" max="25" width="11.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28">

</xml_diff>